<commit_message>
added two more presentations
</commit_message>
<xml_diff>
--- a/topics/projects/Presentations.xlsx
+++ b/topics/projects/Presentations.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ben/Documents/Studies/International Business Management (B. A.)/Data Science and Data Analytics/Projects/Data-Science-and-Data-Analytics/topics/projects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0947A406-ACA7-3D4B-87EB-2791F6AD1504}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74AA8786-CAC5-5143-94C8-4604D46806F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="16860" xr2:uid="{523D878C-183F-FF45-8FEA-63E7989E711F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
   <si>
     <t>Leonie</t>
   </si>
@@ -231,6 +231,45 @@
   </si>
   <si>
     <t>Github + quarto</t>
+  </si>
+  <si>
+    <t>Laurine</t>
+  </si>
+  <si>
+    <t>Eric</t>
+  </si>
+  <si>
+    <t>Mats</t>
+  </si>
+  <si>
+    <t>reading from cards</t>
+  </si>
+  <si>
+    <t>fine, performance, english a bit unsteady</t>
+  </si>
+  <si>
+    <t>description of the data transformation</t>
+  </si>
+  <si>
+    <t>data viz</t>
+  </si>
+  <si>
+    <t>How did you add missing values?</t>
+  </si>
+  <si>
+    <t>why accumulated figures? What did you do with it after?</t>
+  </si>
+  <si>
+    <t>Quarto presentation</t>
+  </si>
+  <si>
+    <t>Hosna</t>
+  </si>
+  <si>
+    <t>How are the datasets connected?</t>
+  </si>
+  <si>
+    <t>reading from cards, monotonic reading</t>
   </si>
 </sst>
 </file>
@@ -998,7 +1037,9 @@
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="1"/>
+      <c r="B5" s="1" t="s">
+        <v>61</v>
+      </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1" t="s">
@@ -1237,8 +1278,12 @@
       <c r="L16" s="1"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
+      <c r="A17" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>62</v>
+      </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
@@ -1248,25 +1293,40 @@
       <c r="I17" s="9"/>
       <c r="J17" s="1"/>
       <c r="K17" s="17"/>
-      <c r="L17" s="12"/>
+      <c r="L17" s="12" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
+      <c r="A18" s="1" t="s">
+        <v>59</v>
+      </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
+      <c r="E18" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="9"/>
-      <c r="J18" s="1"/>
+      <c r="J18" s="1" t="s">
+        <v>66</v>
+      </c>
       <c r="K18" s="17"/>
-      <c r="L18" s="12"/>
+      <c r="L18" s="12" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
+      <c r="A19" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>67</v>
+      </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
@@ -1274,9 +1334,13 @@
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="9"/>
-      <c r="J19" s="1"/>
+      <c r="J19" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="K19" s="17"/>
-      <c r="L19" s="12"/>
+      <c r="L19" s="12" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
@@ -1290,11 +1354,17 @@
       <c r="I20" s="9"/>
       <c r="J20" s="1"/>
       <c r="K20" s="17"/>
-      <c r="L20" s="12"/>
+      <c r="L20" s="12" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
+      <c r="A21" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>70</v>
+      </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
@@ -1302,7 +1372,9 @@
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="9"/>
-      <c r="J21" s="1"/>
+      <c r="J21" s="1" t="s">
+        <v>69</v>
+      </c>
       <c r="K21" s="17"/>
       <c r="L21" s="12"/>
     </row>

</xml_diff>